<commit_message>
Update Kahoot questions to be 100% conceptual (no syntax)
</commit_message>
<xml_diff>
--- a/kahoot_import.xlsx
+++ b/kahoot_import.xlsx
@@ -526,27 +526,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>¿Como funciona JavaScript para ejecutar codigo siendo single-threaded?</t>
+          <t>¿Como se complementan HTML, CSS y JavaScript en una pagina web?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Crea miles de hilos</t>
+          <t>HTML estilos, CSS estructura, JS base de datos</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hace una cosa a la vez pero delega tareas lentas</t>
+          <t>HTML estructura, CSS apariencia, JS interactividad</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Se congela totalmente</t>
+          <t>Los tres hacen exactamente lo mismo</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Duplica la memoria RAM</t>
+          <t>JS solo sirve para diseñar logos</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,31 +561,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>¿En que orden sale: console.log('A'); setTimeout(()=&gt;console.log('B'),0); console.log('C');?</t>
+          <t>¿Como funciona JavaScript para ejecutar tareas siendo de un solo hilo (single-threaded)?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A B C</t>
+          <t>Crea miles de hilos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A C B</t>
+          <t>Hace una cosa a la vez pero delega tareas lentas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B A C</t>
+          <t>Se congela totalmente</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>C B A</t>
+          <t>Duplica la memoria RAM</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -631,27 +631,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>¿Que hace la palabra clave 'await' en: const res = await fetch(url)?</t>
+          <t>¿Que significa que JavaScript sea un lenguaje 'Full-Stack'?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Congela la computadora</t>
+          <t>Solo sirve para computadoras de escritorio</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cancela la peticion</t>
+          <t>Se usa tanto en el navegador (cliente) como en el servidor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Espera la respuesta sin congelar la pagina</t>
+          <t>Solo procesa texto en Word</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Traduce a C++</t>
+          <t>Requiere internet de alta velocidad</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -659,7 +659,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -701,27 +701,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>¿Por que muchos desarrolladores prefieren TypeScript en lugar de JS puro?</t>
+          <t>¿Cual de los siguientes es un framework o libreria popular de JavaScript?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Corre 100x mas rapido</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Detecta errores en el editor ANTES de ejecutar</t>
+          <t>React</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No requiere aprender JS</t>
+          <t>Photoshop</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Elimina las pruebas</t>
+          <t>Windows 11</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -736,27 +736,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>En JavaScript ¿cual es el resultado de ejecutar typeof null?</t>
+          <t>¿Por que muchos desarrolladores prefieren TypeScript en lugar de JS puro?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Corre 100x mas rapido</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>undefined</t>
+          <t>Detecta errores en el editor ANTES de ejecutar</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>No requiere aprender JS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>Elimina las pruebas</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>